<commit_message>
aggiornato con nuovi file e parametri, da tenere per i new var name che se no mi scordo
</commit_message>
<xml_diff>
--- a/WP-2/Data_cleaning/ADNI_variables_cleaned1_COPIA.xlsx
+++ b/WP-2/Data_cleaning/ADNI_variables_cleaned1_COPIA.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ifabfoundation-my.sharepoint.com/personal/chiara_pollicini_ifabfoundation_org/Documents/Documenti/Github/AIND/WP-2/Data_cleaning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{58F97C13-2200-4528-B3C3-FAD4C4233A7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{58F97C13-2200-4528-B3C3-FAD4C4233A7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE3DFDBD-9C9A-4D0B-A1E2-54C2EFEE18FA}"/>
   <bookViews>
-    <workbookView xWindow="-9615" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1350" uniqueCount="218">
   <si>
     <t>file_name</t>
   </si>
@@ -572,6 +585,108 @@
   </si>
   <si>
     <t>DX_YYYY</t>
+  </si>
+  <si>
+    <t>UCSF - ADNI-1 3T Cross-Sectional FreeSurfer (5.1) [ADNI1]</t>
+  </si>
+  <si>
+    <t>UCSFFSX51_ADNI1_3T</t>
+  </si>
+  <si>
+    <t>STATUS</t>
+  </si>
+  <si>
+    <t>ST37SV</t>
+  </si>
+  <si>
+    <t>LVentricle</t>
+  </si>
+  <si>
+    <t>mm3</t>
+  </si>
+  <si>
+    <t>ST10CV</t>
+  </si>
+  <si>
+    <t>ST24CV</t>
+  </si>
+  <si>
+    <t>LEntorhinal</t>
+  </si>
+  <si>
+    <t>ST26CV</t>
+  </si>
+  <si>
+    <t>LFusiform</t>
+  </si>
+  <si>
+    <t>ST29SV</t>
+  </si>
+  <si>
+    <t>Lhippocampus</t>
+  </si>
+  <si>
+    <t>ST40CV</t>
+  </si>
+  <si>
+    <t>LMidTemp</t>
+  </si>
+  <si>
+    <t>ST96SV</t>
+  </si>
+  <si>
+    <t>RVentricle</t>
+  </si>
+  <si>
+    <t>ST83CV</t>
+  </si>
+  <si>
+    <t>Rentorhinal</t>
+  </si>
+  <si>
+    <t>ST85CV</t>
+  </si>
+  <si>
+    <t>RFusiform</t>
+  </si>
+  <si>
+    <t>ST88SV</t>
+  </si>
+  <si>
+    <t>RHippocampus</t>
+  </si>
+  <si>
+    <t>ST99CV</t>
+  </si>
+  <si>
+    <t>RMidTemp</t>
+  </si>
+  <si>
+    <t>UCSF - Cross-Sectional FreeSurfer (5.1) [ADNI1,GO,2]</t>
+  </si>
+  <si>
+    <t>UCSFFSX51</t>
+  </si>
+  <si>
+    <t>UCSFFSX52</t>
+  </si>
+  <si>
+    <t>UCSF - Cross-Sectional FreeSurfer (6.0) [ADNI3]</t>
+  </si>
+  <si>
+    <t>UCSFFSX6</t>
+  </si>
+  <si>
+    <t>UCSF - Cross-Sectional FreeSurfer (7.x) [ADNI1,GO,2,3,4]</t>
+  </si>
+  <si>
+    <t>UCSFFSX7</t>
+  </si>
+  <si>
+    <t>UCSF - Cross-Sectional FreeSurfer (FreeSurfer Version 4.3) [ADNI1,GO,2]</t>
+  </si>
+  <si>
+    <t>UCSFFSX</t>
   </si>
 </sst>
 </file>
@@ -940,10 +1055,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N156"/>
+  <dimension ref="A1:O236"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -959,35 +1074,36 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="1"/>
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1003,11 +1119,11 @@
       <c r="E2" t="s">
         <v>17</v>
       </c>
-      <c r="L2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -1023,11 +1139,11 @@
       <c r="E3" t="s">
         <v>18</v>
       </c>
-      <c r="L3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -1043,11 +1159,11 @@
       <c r="E4" t="s">
         <v>181</v>
       </c>
-      <c r="L4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -1063,11 +1179,11 @@
       <c r="E5" t="s">
         <v>22</v>
       </c>
-      <c r="L5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -1083,11 +1199,11 @@
       <c r="E6" t="s">
         <v>23</v>
       </c>
-      <c r="L6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -1103,14 +1219,14 @@
       <c r="E7" t="s">
         <v>25</v>
       </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7" t="s">
+      <c r="M7">
+        <v>0</v>
+      </c>
+      <c r="N7" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -1126,14 +1242,14 @@
       <c r="E8" t="s">
         <v>104</v>
       </c>
-      <c r="L8">
-        <v>0</v>
-      </c>
-      <c r="M8" t="s">
+      <c r="M8">
+        <v>0</v>
+      </c>
+      <c r="N8" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -1149,14 +1265,14 @@
       <c r="E9" t="s">
         <v>178</v>
       </c>
-      <c r="L9">
-        <v>0</v>
-      </c>
-      <c r="M9" t="s">
+      <c r="M9">
+        <v>0</v>
+      </c>
+      <c r="N9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -1172,14 +1288,14 @@
       <c r="E10" t="s">
         <v>179</v>
       </c>
-      <c r="L10">
-        <v>0</v>
-      </c>
-      <c r="M10" t="s">
+      <c r="M10">
+        <v>0</v>
+      </c>
+      <c r="N10" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -1195,14 +1311,14 @@
       <c r="E11" t="s">
         <v>125</v>
       </c>
-      <c r="L11">
-        <v>0</v>
-      </c>
-      <c r="M11" t="s">
+      <c r="M11">
+        <v>0</v>
+      </c>
+      <c r="N11" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -1218,14 +1334,14 @@
       <c r="E12" t="s">
         <v>180</v>
       </c>
-      <c r="L12">
-        <v>0</v>
-      </c>
-      <c r="M12" t="s">
+      <c r="M12">
+        <v>0</v>
+      </c>
+      <c r="N12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -1241,17 +1357,17 @@
       <c r="E13" t="s">
         <v>37</v>
       </c>
-      <c r="L13">
-        <v>0</v>
-      </c>
-      <c r="M13" t="s">
+      <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="N13" t="s">
         <v>26</v>
       </c>
-      <c r="N13" t="s">
+      <c r="O13" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -1267,17 +1383,17 @@
       <c r="E14" t="s">
         <v>40</v>
       </c>
-      <c r="L14">
+      <c r="M14">
         <v>1</v>
       </c>
-      <c r="M14" t="s">
+      <c r="N14" t="s">
         <v>41</v>
       </c>
-      <c r="N14" t="s">
+      <c r="O14" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -1293,17 +1409,17 @@
       <c r="E15" t="s">
         <v>42</v>
       </c>
-      <c r="L15">
+      <c r="M15">
         <v>1</v>
       </c>
-      <c r="M15" t="s">
+      <c r="N15" t="s">
         <v>41</v>
       </c>
-      <c r="N15" t="s">
+      <c r="O15" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -1319,17 +1435,17 @@
       <c r="E16" t="s">
         <v>44</v>
       </c>
-      <c r="L16">
-        <v>0</v>
-      </c>
-      <c r="M16" t="s">
+      <c r="M16">
+        <v>0</v>
+      </c>
+      <c r="N16" t="s">
         <v>41</v>
       </c>
-      <c r="N16" t="s">
+      <c r="O16" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -1345,17 +1461,17 @@
       <c r="E17" t="s">
         <v>47</v>
       </c>
-      <c r="L17">
-        <v>0</v>
-      </c>
-      <c r="M17" t="s">
+      <c r="M17">
+        <v>0</v>
+      </c>
+      <c r="N17" t="s">
         <v>41</v>
       </c>
-      <c r="N17" t="s">
+      <c r="O17" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>14</v>
       </c>
@@ -1371,17 +1487,17 @@
       <c r="E18" t="s">
         <v>48</v>
       </c>
-      <c r="L18">
-        <v>0</v>
-      </c>
-      <c r="M18" t="s">
+      <c r="M18">
+        <v>0</v>
+      </c>
+      <c r="N18" t="s">
         <v>41</v>
       </c>
-      <c r="N18" t="s">
+      <c r="O18" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>14</v>
       </c>
@@ -1397,17 +1513,17 @@
       <c r="E19" t="s">
         <v>49</v>
       </c>
-      <c r="L19">
-        <v>0</v>
-      </c>
-      <c r="M19" t="s">
+      <c r="M19">
+        <v>0</v>
+      </c>
+      <c r="N19" t="s">
         <v>41</v>
       </c>
-      <c r="N19" t="s">
+      <c r="O19" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>14</v>
       </c>
@@ -1423,17 +1539,17 @@
       <c r="E20" t="s">
         <v>51</v>
       </c>
-      <c r="L20">
-        <v>0</v>
-      </c>
-      <c r="M20" t="s">
+      <c r="M20">
+        <v>0</v>
+      </c>
+      <c r="N20" t="s">
         <v>41</v>
       </c>
-      <c r="N20" t="s">
+      <c r="O20" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>14</v>
       </c>
@@ -1449,17 +1565,17 @@
       <c r="E21" t="s">
         <v>52</v>
       </c>
-      <c r="L21">
-        <v>0</v>
-      </c>
-      <c r="M21" t="s">
+      <c r="M21">
+        <v>0</v>
+      </c>
+      <c r="N21" t="s">
         <v>41</v>
       </c>
-      <c r="N21" t="s">
+      <c r="O21" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>14</v>
       </c>
@@ -1475,17 +1591,17 @@
       <c r="E22" t="s">
         <v>53</v>
       </c>
-      <c r="L22">
+      <c r="M22">
         <v>1</v>
       </c>
-      <c r="M22" t="s">
+      <c r="N22" t="s">
         <v>41</v>
       </c>
-      <c r="N22" t="s">
+      <c r="O22" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>14</v>
       </c>
@@ -1501,17 +1617,17 @@
       <c r="E23" t="s">
         <v>55</v>
       </c>
-      <c r="L23">
+      <c r="M23">
         <v>1</v>
       </c>
-      <c r="M23" t="s">
+      <c r="N23" t="s">
         <v>41</v>
       </c>
-      <c r="N23" t="s">
+      <c r="O23" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>14</v>
       </c>
@@ -1527,17 +1643,17 @@
       <c r="E24" t="s">
         <v>56</v>
       </c>
-      <c r="L24">
+      <c r="M24">
         <v>1</v>
       </c>
-      <c r="M24" t="s">
+      <c r="N24" t="s">
         <v>41</v>
       </c>
-      <c r="N24" t="s">
+      <c r="O24" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>14</v>
       </c>
@@ -1553,17 +1669,17 @@
       <c r="E25" t="s">
         <v>57</v>
       </c>
-      <c r="L25">
+      <c r="M25">
         <v>1</v>
       </c>
-      <c r="M25" t="s">
+      <c r="N25" t="s">
         <v>41</v>
       </c>
-      <c r="N25" t="s">
+      <c r="O25" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>14</v>
       </c>
@@ -1579,17 +1695,17 @@
       <c r="E26" t="s">
         <v>58</v>
       </c>
-      <c r="L26">
+      <c r="M26">
         <v>1</v>
       </c>
-      <c r="M26" t="s">
+      <c r="N26" t="s">
         <v>41</v>
       </c>
-      <c r="N26" t="s">
+      <c r="O26" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>14</v>
       </c>
@@ -1605,17 +1721,17 @@
       <c r="E27" t="s">
         <v>59</v>
       </c>
-      <c r="L27">
+      <c r="M27">
         <v>1</v>
       </c>
-      <c r="M27" t="s">
+      <c r="N27" t="s">
         <v>41</v>
       </c>
-      <c r="N27" t="s">
+      <c r="O27" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>14</v>
       </c>
@@ -1631,17 +1747,17 @@
       <c r="E28" t="s">
         <v>60</v>
       </c>
-      <c r="L28">
+      <c r="M28">
         <v>1</v>
       </c>
-      <c r="M28" t="s">
+      <c r="N28" t="s">
         <v>41</v>
       </c>
-      <c r="N28" t="s">
+      <c r="O28" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>14</v>
       </c>
@@ -1657,14 +1773,14 @@
       <c r="E29" t="s">
         <v>62</v>
       </c>
-      <c r="L29">
-        <v>0</v>
-      </c>
-      <c r="M29" t="s">
+      <c r="M29">
+        <v>0</v>
+      </c>
+      <c r="N29" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>63</v>
       </c>
@@ -1680,11 +1796,11 @@
       <c r="E30" t="s">
         <v>17</v>
       </c>
-      <c r="L30">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>63</v>
       </c>
@@ -1700,11 +1816,11 @@
       <c r="E31" t="s">
         <v>18</v>
       </c>
-      <c r="L31">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>63</v>
       </c>
@@ -1720,11 +1836,11 @@
       <c r="E32" t="s">
         <v>181</v>
       </c>
-      <c r="L32">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>63</v>
       </c>
@@ -1740,11 +1856,11 @@
       <c r="E33" t="s">
         <v>22</v>
       </c>
-      <c r="L33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>63</v>
       </c>
@@ -1760,14 +1876,14 @@
       <c r="E34" t="s">
         <v>178</v>
       </c>
-      <c r="L34">
-        <v>0</v>
-      </c>
-      <c r="M34" t="s">
+      <c r="M34">
+        <v>0</v>
+      </c>
+      <c r="N34" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>63</v>
       </c>
@@ -1783,14 +1899,14 @@
       <c r="E35" t="s">
         <v>179</v>
       </c>
-      <c r="L35">
-        <v>0</v>
-      </c>
-      <c r="M35" t="s">
+      <c r="M35">
+        <v>0</v>
+      </c>
+      <c r="N35" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>63</v>
       </c>
@@ -1806,14 +1922,14 @@
       <c r="E36" t="s">
         <v>125</v>
       </c>
-      <c r="L36">
-        <v>0</v>
-      </c>
-      <c r="M36" t="s">
+      <c r="M36">
+        <v>0</v>
+      </c>
+      <c r="N36" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>63</v>
       </c>
@@ -1829,14 +1945,14 @@
       <c r="E37" t="s">
         <v>104</v>
       </c>
-      <c r="L37">
-        <v>0</v>
-      </c>
-      <c r="M37" t="s">
+      <c r="M37">
+        <v>0</v>
+      </c>
+      <c r="N37" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>63</v>
       </c>
@@ -1852,17 +1968,17 @@
       <c r="E38" t="s">
         <v>73</v>
       </c>
-      <c r="L38">
-        <v>0</v>
-      </c>
-      <c r="M38" t="s">
+      <c r="M38">
+        <v>0</v>
+      </c>
+      <c r="N38" t="s">
         <v>41</v>
       </c>
-      <c r="N38" t="s">
+      <c r="O38" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>63</v>
       </c>
@@ -1878,11 +1994,11 @@
       <c r="E39" t="s">
         <v>74</v>
       </c>
-      <c r="L39">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>63</v>
       </c>
@@ -1898,17 +2014,17 @@
       <c r="E40" t="s">
         <v>75</v>
       </c>
-      <c r="L40">
-        <v>0</v>
-      </c>
-      <c r="M40" t="s">
+      <c r="M40">
+        <v>0</v>
+      </c>
+      <c r="N40" t="s">
         <v>41</v>
       </c>
-      <c r="N40" t="s">
+      <c r="O40" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>63</v>
       </c>
@@ -1924,14 +2040,14 @@
       <c r="E41" t="s">
         <v>62</v>
       </c>
-      <c r="L41">
-        <v>0</v>
-      </c>
-      <c r="M41" t="s">
+      <c r="M41">
+        <v>0</v>
+      </c>
+      <c r="N41" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>63</v>
       </c>
@@ -1947,17 +2063,17 @@
       <c r="E42" t="s">
         <v>77</v>
       </c>
-      <c r="L42">
-        <v>0</v>
-      </c>
-      <c r="M42" t="s">
+      <c r="M42">
+        <v>0</v>
+      </c>
+      <c r="N42" t="s">
         <v>41</v>
       </c>
-      <c r="N42" t="s">
+      <c r="O42" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>63</v>
       </c>
@@ -1973,17 +2089,17 @@
       <c r="E43" t="s">
         <v>78</v>
       </c>
-      <c r="L43">
-        <v>0</v>
-      </c>
-      <c r="M43" t="s">
+      <c r="M43">
+        <v>0</v>
+      </c>
+      <c r="N43" t="s">
         <v>41</v>
       </c>
-      <c r="N43" t="s">
+      <c r="O43" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>63</v>
       </c>
@@ -1999,17 +2115,17 @@
       <c r="E44" t="s">
         <v>79</v>
       </c>
-      <c r="L44">
-        <v>0</v>
-      </c>
-      <c r="M44" t="s">
+      <c r="M44">
+        <v>0</v>
+      </c>
+      <c r="N44" t="s">
         <v>41</v>
       </c>
-      <c r="N44" t="s">
+      <c r="O44" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>63</v>
       </c>
@@ -2025,14 +2141,14 @@
       <c r="E45" t="s">
         <v>81</v>
       </c>
-      <c r="L45">
-        <v>0</v>
-      </c>
-      <c r="M45" t="s">
+      <c r="M45">
+        <v>0</v>
+      </c>
+      <c r="N45" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>63</v>
       </c>
@@ -2048,14 +2164,14 @@
       <c r="E46" t="s">
         <v>25</v>
       </c>
-      <c r="L46">
-        <v>0</v>
-      </c>
-      <c r="M46" t="s">
+      <c r="M46">
+        <v>0</v>
+      </c>
+      <c r="N46" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>83</v>
       </c>
@@ -2072,7 +2188,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>83</v>
       </c>
@@ -2633,7 +2749,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>83</v>
       </c>
@@ -2650,7 +2766,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>83</v>
       </c>
@@ -2667,7 +2783,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>83</v>
       </c>
@@ -2684,7 +2800,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>83</v>
       </c>
@@ -2701,7 +2817,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>83</v>
       </c>
@@ -2718,7 +2834,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>83</v>
       </c>
@@ -2735,7 +2851,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>83</v>
       </c>
@@ -2752,7 +2868,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>83</v>
       </c>
@@ -2769,7 +2885,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>83</v>
       </c>
@@ -2786,7 +2902,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>83</v>
       </c>
@@ -2803,7 +2919,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>128</v>
       </c>
@@ -2819,11 +2935,11 @@
       <c r="E91" t="s">
         <v>17</v>
       </c>
-      <c r="L91">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>128</v>
       </c>
@@ -2839,11 +2955,11 @@
       <c r="E92" t="s">
         <v>181</v>
       </c>
-      <c r="L92">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>128</v>
       </c>
@@ -2859,11 +2975,11 @@
       <c r="E93" t="s">
         <v>18</v>
       </c>
-      <c r="L93">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>128</v>
       </c>
@@ -2879,11 +2995,11 @@
       <c r="E94" t="s">
         <v>22</v>
       </c>
-      <c r="L94">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M94">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>128</v>
       </c>
@@ -2899,11 +3015,11 @@
       <c r="E95" t="s">
         <v>23</v>
       </c>
-      <c r="L95">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M95">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>128</v>
       </c>
@@ -2919,11 +3035,11 @@
       <c r="E96" t="s">
         <v>62</v>
       </c>
-      <c r="L96">
+      <c r="M96">
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>128</v>
       </c>
@@ -2939,17 +3055,17 @@
       <c r="E97" t="s">
         <v>46</v>
       </c>
-      <c r="L97">
-        <v>0</v>
-      </c>
-      <c r="M97" t="s">
+      <c r="M97">
+        <v>0</v>
+      </c>
+      <c r="N97" t="s">
         <v>41</v>
       </c>
-      <c r="N97" t="s">
+      <c r="O97" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="98" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>128</v>
       </c>
@@ -2965,17 +3081,17 @@
       <c r="E98" t="s">
         <v>49</v>
       </c>
-      <c r="L98">
-        <v>0</v>
-      </c>
-      <c r="M98" t="s">
+      <c r="M98">
+        <v>0</v>
+      </c>
+      <c r="N98" t="s">
         <v>41</v>
       </c>
-      <c r="N98" t="s">
+      <c r="O98" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="99" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>128</v>
       </c>
@@ -2991,17 +3107,17 @@
       <c r="E99" t="s">
         <v>182</v>
       </c>
-      <c r="L99">
-        <v>0</v>
-      </c>
-      <c r="M99" t="s">
+      <c r="M99">
+        <v>0</v>
+      </c>
+      <c r="N99" t="s">
         <v>41</v>
       </c>
-      <c r="N99" t="s">
+      <c r="O99" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="100" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>128</v>
       </c>
@@ -3017,17 +3133,17 @@
       <c r="E100" t="s">
         <v>134</v>
       </c>
-      <c r="L100">
-        <v>0</v>
-      </c>
-      <c r="M100" t="s">
+      <c r="M100">
+        <v>0</v>
+      </c>
+      <c r="N100" t="s">
         <v>41</v>
       </c>
-      <c r="N100" t="s">
+      <c r="O100" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="101" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>128</v>
       </c>
@@ -3043,14 +3159,14 @@
       <c r="E101" t="s">
         <v>135</v>
       </c>
-      <c r="L101">
-        <v>0</v>
-      </c>
-      <c r="M101" t="s">
+      <c r="M101">
+        <v>0</v>
+      </c>
+      <c r="N101" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="102" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>128</v>
       </c>
@@ -3066,14 +3182,14 @@
       <c r="E102" t="s">
         <v>136</v>
       </c>
-      <c r="L102">
-        <v>0</v>
-      </c>
-      <c r="M102" t="s">
+      <c r="M102">
+        <v>0</v>
+      </c>
+      <c r="N102" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="103" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>128</v>
       </c>
@@ -3089,17 +3205,17 @@
       <c r="E103" t="s">
         <v>52</v>
       </c>
-      <c r="L103">
-        <v>0</v>
-      </c>
-      <c r="M103" t="s">
+      <c r="M103">
+        <v>0</v>
+      </c>
+      <c r="N103" t="s">
         <v>41</v>
       </c>
-      <c r="N103" t="s">
+      <c r="O103" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="104" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>128</v>
       </c>
@@ -3115,14 +3231,14 @@
       <c r="E104" t="s">
         <v>138</v>
       </c>
-      <c r="L104">
-        <v>0</v>
-      </c>
-      <c r="M104" t="s">
+      <c r="M104">
+        <v>0</v>
+      </c>
+      <c r="N104" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="105" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>128</v>
       </c>
@@ -3138,14 +3254,14 @@
       <c r="E105" t="s">
         <v>139</v>
       </c>
-      <c r="L105">
-        <v>0</v>
-      </c>
-      <c r="M105" t="s">
+      <c r="M105">
+        <v>0</v>
+      </c>
+      <c r="N105" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="106" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>128</v>
       </c>
@@ -3161,17 +3277,17 @@
       <c r="E106" t="s">
         <v>43</v>
       </c>
-      <c r="L106">
-        <v>0</v>
-      </c>
-      <c r="M106" t="s">
+      <c r="M106">
+        <v>0</v>
+      </c>
+      <c r="N106" t="s">
         <v>41</v>
       </c>
-      <c r="N106" t="s">
+      <c r="O106" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="107" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>141</v>
       </c>
@@ -3187,11 +3303,11 @@
       <c r="E107" t="s">
         <v>17</v>
       </c>
-      <c r="L107">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="108" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M107">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>141</v>
       </c>
@@ -3207,11 +3323,11 @@
       <c r="E108" t="s">
         <v>181</v>
       </c>
-      <c r="L108">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="109" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M108">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>141</v>
       </c>
@@ -3227,11 +3343,11 @@
       <c r="E109" t="s">
         <v>18</v>
       </c>
-      <c r="L109">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="110" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M109">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>141</v>
       </c>
@@ -3247,11 +3363,11 @@
       <c r="E110" t="s">
         <v>143</v>
       </c>
-      <c r="L110">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="111" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M110">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>141</v>
       </c>
@@ -3267,11 +3383,11 @@
       <c r="E111" t="s">
         <v>104</v>
       </c>
-      <c r="L111">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="112" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M111">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>141</v>
       </c>
@@ -3287,11 +3403,11 @@
       <c r="E112" t="s">
         <v>144</v>
       </c>
-      <c r="L112">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="113" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M112">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>141</v>
       </c>
@@ -3307,14 +3423,14 @@
       <c r="E113" t="s">
         <v>180</v>
       </c>
-      <c r="L113">
-        <v>0</v>
-      </c>
-      <c r="M113" t="s">
+      <c r="M113">
+        <v>0</v>
+      </c>
+      <c r="N113" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="114" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>141</v>
       </c>
@@ -3330,14 +3446,14 @@
       <c r="E114" t="s">
         <v>178</v>
       </c>
-      <c r="L114">
-        <v>0</v>
-      </c>
-      <c r="M114" t="s">
+      <c r="M114">
+        <v>0</v>
+      </c>
+      <c r="N114" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="115" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>141</v>
       </c>
@@ -3353,14 +3469,14 @@
       <c r="E115" t="s">
         <v>145</v>
       </c>
-      <c r="L115">
+      <c r="M115">
         <v>1</v>
       </c>
-      <c r="M115" t="s">
+      <c r="N115" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="116" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>141</v>
       </c>
@@ -3376,14 +3492,14 @@
       <c r="E116" t="s">
         <v>179</v>
       </c>
-      <c r="L116">
-        <v>0</v>
-      </c>
-      <c r="M116" t="s">
+      <c r="M116">
+        <v>0</v>
+      </c>
+      <c r="N116" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="117" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>141</v>
       </c>
@@ -3399,14 +3515,14 @@
       <c r="E117" t="s">
         <v>125</v>
       </c>
-      <c r="L117">
-        <v>0</v>
-      </c>
-      <c r="M117" t="s">
+      <c r="M117">
+        <v>0</v>
+      </c>
+      <c r="N117" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="118" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>146</v>
       </c>
@@ -3422,11 +3538,11 @@
       <c r="E118" t="s">
         <v>22</v>
       </c>
-      <c r="L118">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="119" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M118">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>146</v>
       </c>
@@ -3442,14 +3558,14 @@
       <c r="E119" t="s">
         <v>147</v>
       </c>
-      <c r="L119">
-        <v>0</v>
-      </c>
-      <c r="M119" t="s">
+      <c r="M119">
+        <v>0</v>
+      </c>
+      <c r="N119" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="120" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>146</v>
       </c>
@@ -3465,11 +3581,11 @@
       <c r="E120" t="s">
         <v>148</v>
       </c>
-      <c r="L120">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="121" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M120">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>146</v>
       </c>
@@ -3485,14 +3601,14 @@
       <c r="E121" t="s">
         <v>183</v>
       </c>
-      <c r="L121">
+      <c r="M121">
         <v>1</v>
       </c>
-      <c r="M121" t="s">
+      <c r="N121" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="122" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>150</v>
       </c>
@@ -3508,14 +3624,14 @@
       <c r="E122" t="s">
         <v>17</v>
       </c>
-      <c r="L122">
-        <v>0</v>
-      </c>
-      <c r="M122" t="s">
+      <c r="M122">
+        <v>0</v>
+      </c>
+      <c r="N122" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="123" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>150</v>
       </c>
@@ -3531,14 +3647,14 @@
       <c r="E123" t="s">
         <v>181</v>
       </c>
-      <c r="L123">
-        <v>0</v>
-      </c>
-      <c r="M123" t="s">
+      <c r="M123">
+        <v>0</v>
+      </c>
+      <c r="N123" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="124" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>150</v>
       </c>
@@ -3554,11 +3670,11 @@
       <c r="E124" t="s">
         <v>18</v>
       </c>
-      <c r="L124">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="125" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M124">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>150</v>
       </c>
@@ -3574,11 +3690,11 @@
       <c r="E125" t="s">
         <v>143</v>
       </c>
-      <c r="L125">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="126" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M125">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>150</v>
       </c>
@@ -3594,14 +3710,14 @@
       <c r="E126" t="s">
         <v>49</v>
       </c>
-      <c r="L126">
-        <v>0</v>
-      </c>
-      <c r="N126" t="s">
+      <c r="M126">
+        <v>0</v>
+      </c>
+      <c r="O126" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="127" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>150</v>
       </c>
@@ -3617,11 +3733,11 @@
       <c r="E127" t="s">
         <v>22</v>
       </c>
-      <c r="L127">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="128" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M127">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>152</v>
       </c>
@@ -3637,14 +3753,14 @@
       <c r="E128" t="s">
         <v>17</v>
       </c>
-      <c r="L128">
-        <v>0</v>
-      </c>
-      <c r="M128" t="s">
+      <c r="M128">
+        <v>0</v>
+      </c>
+      <c r="N128" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="129" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>152</v>
       </c>
@@ -3660,11 +3776,11 @@
       <c r="E129" t="s">
         <v>181</v>
       </c>
-      <c r="L129">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="130" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="M129">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>152</v>
       </c>
@@ -3680,11 +3796,11 @@
       <c r="E130" t="s">
         <v>18</v>
       </c>
-      <c r="L130">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="131" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="M130">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>152</v>
       </c>
@@ -3700,11 +3816,11 @@
       <c r="E131" t="s">
         <v>23</v>
       </c>
-      <c r="L131">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="132" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="M131">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>152</v>
       </c>
@@ -3720,14 +3836,14 @@
       <c r="E132" t="s">
         <v>154</v>
       </c>
-      <c r="L132">
+      <c r="M132">
         <v>1</v>
       </c>
-      <c r="M132" t="s">
+      <c r="N132" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="133" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>152</v>
       </c>
@@ -3743,14 +3859,14 @@
       <c r="E133" t="s">
         <v>155</v>
       </c>
-      <c r="L133">
+      <c r="M133">
         <v>1</v>
       </c>
-      <c r="M133" t="s">
+      <c r="N133" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="134" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>152</v>
       </c>
@@ -3766,14 +3882,14 @@
       <c r="E134" t="s">
         <v>156</v>
       </c>
-      <c r="L134">
+      <c r="M134">
         <v>1</v>
       </c>
-      <c r="M134" t="s">
+      <c r="N134" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="135" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>152</v>
       </c>
@@ -3789,14 +3905,14 @@
       <c r="E135" t="s">
         <v>157</v>
       </c>
-      <c r="L135">
-        <v>0</v>
-      </c>
-      <c r="M135" t="s">
+      <c r="M135">
+        <v>0</v>
+      </c>
+      <c r="N135" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="136" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>152</v>
       </c>
@@ -3812,14 +3928,14 @@
       <c r="E136" t="s">
         <v>158</v>
       </c>
-      <c r="L136">
+      <c r="M136">
         <v>1</v>
       </c>
-      <c r="M136" t="s">
+      <c r="N136" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="137" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>152</v>
       </c>
@@ -3835,14 +3951,14 @@
       <c r="E137" t="s">
         <v>159</v>
       </c>
-      <c r="L137">
+      <c r="M137">
         <v>1</v>
       </c>
-      <c r="M137" t="s">
+      <c r="N137" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="138" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>152</v>
       </c>
@@ -3858,14 +3974,14 @@
       <c r="E138" t="s">
         <v>160</v>
       </c>
-      <c r="L138">
+      <c r="M138">
         <v>1</v>
       </c>
-      <c r="M138" t="s">
+      <c r="N138" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="139" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>152</v>
       </c>
@@ -3881,14 +3997,14 @@
       <c r="E139" t="s">
         <v>161</v>
       </c>
-      <c r="L139">
+      <c r="M139">
         <v>1</v>
       </c>
-      <c r="M139" t="s">
+      <c r="N139" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="140" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>152</v>
       </c>
@@ -3904,14 +4020,14 @@
       <c r="E140" t="s">
         <v>162</v>
       </c>
-      <c r="L140">
+      <c r="M140">
         <v>1</v>
       </c>
-      <c r="M140" t="s">
+      <c r="N140" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="141" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>152</v>
       </c>
@@ -3927,14 +4043,14 @@
       <c r="E141" t="s">
         <v>163</v>
       </c>
-      <c r="L141">
+      <c r="M141">
         <v>1</v>
       </c>
-      <c r="M141" t="s">
+      <c r="N141" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="142" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>152</v>
       </c>
@@ -3950,14 +4066,14 @@
       <c r="E142" t="s">
         <v>164</v>
       </c>
-      <c r="L142">
+      <c r="M142">
         <v>1</v>
       </c>
-      <c r="M142" t="s">
+      <c r="N142" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="143" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>152</v>
       </c>
@@ -3973,14 +4089,14 @@
       <c r="E143" t="s">
         <v>165</v>
       </c>
-      <c r="L143">
-        <v>0</v>
-      </c>
-      <c r="M143" t="s">
+      <c r="M143">
+        <v>0</v>
+      </c>
+      <c r="N143" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="144" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>152</v>
       </c>
@@ -3996,14 +4112,14 @@
       <c r="E144" t="s">
         <v>166</v>
       </c>
-      <c r="L144">
+      <c r="M144">
         <v>1</v>
       </c>
-      <c r="M144" t="s">
+      <c r="N144" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>152</v>
       </c>
@@ -4019,14 +4135,14 @@
       <c r="E145" t="s">
         <v>167</v>
       </c>
-      <c r="L145">
+      <c r="M145">
         <v>1</v>
       </c>
-      <c r="M145" t="s">
+      <c r="N145" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>152</v>
       </c>
@@ -4042,14 +4158,14 @@
       <c r="E146" t="s">
         <v>168</v>
       </c>
-      <c r="L146">
+      <c r="M146">
         <v>1</v>
       </c>
-      <c r="M146" t="s">
+      <c r="N146" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>152</v>
       </c>
@@ -4065,14 +4181,14 @@
       <c r="E147" t="s">
         <v>169</v>
       </c>
-      <c r="L147">
+      <c r="M147">
         <v>1</v>
       </c>
-      <c r="M147" t="s">
+      <c r="N147" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>152</v>
       </c>
@@ -4088,14 +4204,14 @@
       <c r="E148" t="s">
         <v>170</v>
       </c>
-      <c r="L148">
-        <v>0</v>
-      </c>
-      <c r="M148" t="s">
+      <c r="M148">
+        <v>0</v>
+      </c>
+      <c r="N148" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>152</v>
       </c>
@@ -4111,14 +4227,14 @@
       <c r="E149" t="s">
         <v>171</v>
       </c>
-      <c r="L149">
+      <c r="M149">
         <v>1</v>
       </c>
-      <c r="M149" t="s">
+      <c r="N149" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>152</v>
       </c>
@@ -4134,14 +4250,14 @@
       <c r="E150" t="s">
         <v>172</v>
       </c>
-      <c r="L150">
+      <c r="M150">
         <v>1</v>
       </c>
-      <c r="M150" t="s">
+      <c r="N150" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>152</v>
       </c>
@@ -4157,14 +4273,14 @@
       <c r="E151" t="s">
         <v>173</v>
       </c>
-      <c r="L151">
+      <c r="M151">
         <v>1</v>
       </c>
-      <c r="M151" t="s">
+      <c r="N151" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>152</v>
       </c>
@@ -4180,14 +4296,14 @@
       <c r="E152" t="s">
         <v>174</v>
       </c>
-      <c r="L152">
+      <c r="M152">
         <v>1</v>
       </c>
-      <c r="M152" t="s">
+      <c r="N152" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>152</v>
       </c>
@@ -4203,14 +4319,14 @@
       <c r="E153" t="s">
         <v>175</v>
       </c>
-      <c r="L153">
+      <c r="M153">
         <v>1</v>
       </c>
-      <c r="M153" t="s">
+      <c r="N153" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>152</v>
       </c>
@@ -4226,11 +4342,11 @@
       <c r="E154" t="s">
         <v>67</v>
       </c>
-      <c r="L154">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="M154">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>152</v>
       </c>
@@ -4246,14 +4362,14 @@
       <c r="E155" t="s">
         <v>176</v>
       </c>
-      <c r="L155">
+      <c r="M155">
         <v>1</v>
       </c>
-      <c r="M155" t="s">
+      <c r="N155" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>152</v>
       </c>
@@ -4269,11 +4385,1533 @@
       <c r="E156" t="s">
         <v>62</v>
       </c>
-      <c r="L156">
-        <v>0</v>
-      </c>
-      <c r="M156" t="s">
+      <c r="M156">
+        <v>0</v>
+      </c>
+      <c r="N156" t="s">
         <v>41</v>
+      </c>
+    </row>
+    <row r="157" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A157" t="s">
+        <v>184</v>
+      </c>
+      <c r="B157" t="s">
+        <v>185</v>
+      </c>
+      <c r="C157" t="s">
+        <v>16</v>
+      </c>
+      <c r="D157" t="s">
+        <v>18</v>
+      </c>
+      <c r="E157" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="158" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A158" t="s">
+        <v>184</v>
+      </c>
+      <c r="B158" t="s">
+        <v>185</v>
+      </c>
+      <c r="C158" t="s">
+        <v>66</v>
+      </c>
+      <c r="D158" t="s">
+        <v>22</v>
+      </c>
+      <c r="E158" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="159" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A159" t="s">
+        <v>184</v>
+      </c>
+      <c r="B159" t="s">
+        <v>185</v>
+      </c>
+      <c r="C159" t="s">
+        <v>66</v>
+      </c>
+      <c r="D159" t="s">
+        <v>23</v>
+      </c>
+      <c r="E159" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="160" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A160" t="s">
+        <v>184</v>
+      </c>
+      <c r="B160" t="s">
+        <v>185</v>
+      </c>
+      <c r="C160" t="s">
+        <v>89</v>
+      </c>
+      <c r="D160" t="s">
+        <v>186</v>
+      </c>
+      <c r="E160" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A161" t="s">
+        <v>184</v>
+      </c>
+      <c r="B161" t="s">
+        <v>185</v>
+      </c>
+      <c r="C161" t="s">
+        <v>54</v>
+      </c>
+      <c r="D161" t="s">
+        <v>187</v>
+      </c>
+      <c r="E161" t="s">
+        <v>188</v>
+      </c>
+      <c r="F161" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A162" t="s">
+        <v>184</v>
+      </c>
+      <c r="B162" t="s">
+        <v>185</v>
+      </c>
+      <c r="C162" t="s">
+        <v>54</v>
+      </c>
+      <c r="D162" t="s">
+        <v>190</v>
+      </c>
+      <c r="E162" t="s">
+        <v>60</v>
+      </c>
+      <c r="F162" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A163" t="s">
+        <v>184</v>
+      </c>
+      <c r="B163" t="s">
+        <v>185</v>
+      </c>
+      <c r="C163" t="s">
+        <v>54</v>
+      </c>
+      <c r="D163" t="s">
+        <v>191</v>
+      </c>
+      <c r="E163" t="s">
+        <v>192</v>
+      </c>
+      <c r="F163" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A164" t="s">
+        <v>184</v>
+      </c>
+      <c r="B164" t="s">
+        <v>185</v>
+      </c>
+      <c r="C164" t="s">
+        <v>54</v>
+      </c>
+      <c r="D164" t="s">
+        <v>193</v>
+      </c>
+      <c r="E164" t="s">
+        <v>194</v>
+      </c>
+      <c r="F164" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A165" t="s">
+        <v>184</v>
+      </c>
+      <c r="B165" t="s">
+        <v>185</v>
+      </c>
+      <c r="C165" t="s">
+        <v>54</v>
+      </c>
+      <c r="D165" t="s">
+        <v>195</v>
+      </c>
+      <c r="E165" t="s">
+        <v>196</v>
+      </c>
+      <c r="F165" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A166" t="s">
+        <v>184</v>
+      </c>
+      <c r="B166" t="s">
+        <v>185</v>
+      </c>
+      <c r="C166" t="s">
+        <v>54</v>
+      </c>
+      <c r="D166" t="s">
+        <v>197</v>
+      </c>
+      <c r="E166" t="s">
+        <v>198</v>
+      </c>
+      <c r="F166" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A167" t="s">
+        <v>184</v>
+      </c>
+      <c r="B167" t="s">
+        <v>185</v>
+      </c>
+      <c r="C167" t="s">
+        <v>54</v>
+      </c>
+      <c r="D167" t="s">
+        <v>199</v>
+      </c>
+      <c r="E167" t="s">
+        <v>200</v>
+      </c>
+      <c r="F167" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A168" t="s">
+        <v>184</v>
+      </c>
+      <c r="B168" t="s">
+        <v>185</v>
+      </c>
+      <c r="C168" t="s">
+        <v>54</v>
+      </c>
+      <c r="D168" t="s">
+        <v>201</v>
+      </c>
+      <c r="E168" t="s">
+        <v>202</v>
+      </c>
+      <c r="F168" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="169" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A169" t="s">
+        <v>184</v>
+      </c>
+      <c r="B169" t="s">
+        <v>185</v>
+      </c>
+      <c r="C169" t="s">
+        <v>54</v>
+      </c>
+      <c r="D169" t="s">
+        <v>203</v>
+      </c>
+      <c r="E169" t="s">
+        <v>204</v>
+      </c>
+      <c r="F169" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="170" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A170" t="s">
+        <v>184</v>
+      </c>
+      <c r="B170" t="s">
+        <v>185</v>
+      </c>
+      <c r="C170" t="s">
+        <v>54</v>
+      </c>
+      <c r="D170" t="s">
+        <v>205</v>
+      </c>
+      <c r="E170" t="s">
+        <v>206</v>
+      </c>
+      <c r="F170" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="171" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A171" t="s">
+        <v>184</v>
+      </c>
+      <c r="B171" t="s">
+        <v>185</v>
+      </c>
+      <c r="C171" t="s">
+        <v>54</v>
+      </c>
+      <c r="D171" t="s">
+        <v>207</v>
+      </c>
+      <c r="E171" t="s">
+        <v>208</v>
+      </c>
+      <c r="F171" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="172" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A172" t="s">
+        <v>209</v>
+      </c>
+      <c r="B172" t="s">
+        <v>210</v>
+      </c>
+      <c r="C172" t="s">
+        <v>16</v>
+      </c>
+      <c r="D172" t="s">
+        <v>18</v>
+      </c>
+      <c r="E172" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A173" t="s">
+        <v>209</v>
+      </c>
+      <c r="B173" t="s">
+        <v>210</v>
+      </c>
+      <c r="C173" t="s">
+        <v>66</v>
+      </c>
+      <c r="D173" t="s">
+        <v>22</v>
+      </c>
+      <c r="E173" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="174" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A174" t="s">
+        <v>209</v>
+      </c>
+      <c r="B174" t="s">
+        <v>210</v>
+      </c>
+      <c r="C174" t="s">
+        <v>66</v>
+      </c>
+      <c r="D174" t="s">
+        <v>67</v>
+      </c>
+      <c r="E174" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="175" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A175" t="s">
+        <v>209</v>
+      </c>
+      <c r="B175" t="s">
+        <v>210</v>
+      </c>
+      <c r="C175" t="s">
+        <v>66</v>
+      </c>
+      <c r="D175" t="s">
+        <v>23</v>
+      </c>
+      <c r="E175" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="176" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A176" t="s">
+        <v>209</v>
+      </c>
+      <c r="B176" t="s">
+        <v>211</v>
+      </c>
+      <c r="C176" t="s">
+        <v>89</v>
+      </c>
+      <c r="D176" t="s">
+        <v>186</v>
+      </c>
+      <c r="E176" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="177" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A177" t="s">
+        <v>209</v>
+      </c>
+      <c r="B177" t="s">
+        <v>210</v>
+      </c>
+      <c r="C177" t="s">
+        <v>54</v>
+      </c>
+      <c r="D177" t="s">
+        <v>187</v>
+      </c>
+      <c r="E177" t="s">
+        <v>188</v>
+      </c>
+      <c r="F177" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="178" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A178" t="s">
+        <v>209</v>
+      </c>
+      <c r="B178" t="s">
+        <v>210</v>
+      </c>
+      <c r="C178" t="s">
+        <v>54</v>
+      </c>
+      <c r="D178" t="s">
+        <v>190</v>
+      </c>
+      <c r="E178" t="s">
+        <v>60</v>
+      </c>
+      <c r="F178" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="179" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A179" t="s">
+        <v>209</v>
+      </c>
+      <c r="B179" t="s">
+        <v>210</v>
+      </c>
+      <c r="C179" t="s">
+        <v>54</v>
+      </c>
+      <c r="D179" t="s">
+        <v>191</v>
+      </c>
+      <c r="E179" t="s">
+        <v>192</v>
+      </c>
+      <c r="F179" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="180" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A180" t="s">
+        <v>209</v>
+      </c>
+      <c r="B180" t="s">
+        <v>210</v>
+      </c>
+      <c r="C180" t="s">
+        <v>54</v>
+      </c>
+      <c r="D180" t="s">
+        <v>193</v>
+      </c>
+      <c r="E180" t="s">
+        <v>194</v>
+      </c>
+      <c r="F180" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A181" t="s">
+        <v>209</v>
+      </c>
+      <c r="B181" t="s">
+        <v>210</v>
+      </c>
+      <c r="C181" t="s">
+        <v>54</v>
+      </c>
+      <c r="D181" t="s">
+        <v>195</v>
+      </c>
+      <c r="E181" t="s">
+        <v>196</v>
+      </c>
+      <c r="F181" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="182" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A182" t="s">
+        <v>209</v>
+      </c>
+      <c r="B182" t="s">
+        <v>210</v>
+      </c>
+      <c r="C182" t="s">
+        <v>54</v>
+      </c>
+      <c r="D182" t="s">
+        <v>197</v>
+      </c>
+      <c r="E182" t="s">
+        <v>198</v>
+      </c>
+      <c r="F182" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="183" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A183" t="s">
+        <v>209</v>
+      </c>
+      <c r="B183" t="s">
+        <v>210</v>
+      </c>
+      <c r="C183" t="s">
+        <v>54</v>
+      </c>
+      <c r="D183" t="s">
+        <v>199</v>
+      </c>
+      <c r="E183" t="s">
+        <v>200</v>
+      </c>
+      <c r="F183" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="184" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A184" t="s">
+        <v>209</v>
+      </c>
+      <c r="B184" t="s">
+        <v>210</v>
+      </c>
+      <c r="C184" t="s">
+        <v>54</v>
+      </c>
+      <c r="D184" t="s">
+        <v>201</v>
+      </c>
+      <c r="E184" t="s">
+        <v>202</v>
+      </c>
+      <c r="F184" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="185" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A185" t="s">
+        <v>209</v>
+      </c>
+      <c r="B185" t="s">
+        <v>210</v>
+      </c>
+      <c r="C185" t="s">
+        <v>54</v>
+      </c>
+      <c r="D185" t="s">
+        <v>203</v>
+      </c>
+      <c r="E185" t="s">
+        <v>204</v>
+      </c>
+      <c r="F185" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="186" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A186" t="s">
+        <v>209</v>
+      </c>
+      <c r="B186" t="s">
+        <v>210</v>
+      </c>
+      <c r="C186" t="s">
+        <v>54</v>
+      </c>
+      <c r="D186" t="s">
+        <v>205</v>
+      </c>
+      <c r="E186" t="s">
+        <v>206</v>
+      </c>
+      <c r="F186" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="187" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A187" t="s">
+        <v>209</v>
+      </c>
+      <c r="B187" t="s">
+        <v>210</v>
+      </c>
+      <c r="C187" t="s">
+        <v>54</v>
+      </c>
+      <c r="D187" t="s">
+        <v>207</v>
+      </c>
+      <c r="E187" t="s">
+        <v>208</v>
+      </c>
+      <c r="F187" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="188" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A188" t="s">
+        <v>212</v>
+      </c>
+      <c r="B188" t="s">
+        <v>213</v>
+      </c>
+      <c r="C188" t="s">
+        <v>16</v>
+      </c>
+      <c r="D188" t="s">
+        <v>18</v>
+      </c>
+      <c r="E188" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="189" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A189" t="s">
+        <v>212</v>
+      </c>
+      <c r="B189" t="s">
+        <v>213</v>
+      </c>
+      <c r="C189" t="s">
+        <v>19</v>
+      </c>
+      <c r="D189" t="s">
+        <v>65</v>
+      </c>
+      <c r="E189" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="190" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A190" t="s">
+        <v>212</v>
+      </c>
+      <c r="B190" t="s">
+        <v>213</v>
+      </c>
+      <c r="C190" t="s">
+        <v>66</v>
+      </c>
+      <c r="D190" t="s">
+        <v>22</v>
+      </c>
+      <c r="E190" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A191" t="s">
+        <v>212</v>
+      </c>
+      <c r="B191" t="s">
+        <v>213</v>
+      </c>
+      <c r="C191" t="s">
+        <v>66</v>
+      </c>
+      <c r="D191" t="s">
+        <v>67</v>
+      </c>
+      <c r="E191" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="192" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A192" t="s">
+        <v>212</v>
+      </c>
+      <c r="B192" t="s">
+        <v>213</v>
+      </c>
+      <c r="C192" t="s">
+        <v>66</v>
+      </c>
+      <c r="D192" t="s">
+        <v>23</v>
+      </c>
+      <c r="E192" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="193" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A193" t="s">
+        <v>212</v>
+      </c>
+      <c r="B193" t="s">
+        <v>213</v>
+      </c>
+      <c r="C193" t="s">
+        <v>89</v>
+      </c>
+      <c r="D193" t="s">
+        <v>186</v>
+      </c>
+      <c r="E193" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="194" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A194" t="s">
+        <v>212</v>
+      </c>
+      <c r="B194" t="s">
+        <v>213</v>
+      </c>
+      <c r="C194" t="s">
+        <v>54</v>
+      </c>
+      <c r="D194" t="s">
+        <v>187</v>
+      </c>
+      <c r="E194" t="s">
+        <v>188</v>
+      </c>
+      <c r="F194" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="195" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A195" t="s">
+        <v>212</v>
+      </c>
+      <c r="B195" t="s">
+        <v>213</v>
+      </c>
+      <c r="C195" t="s">
+        <v>54</v>
+      </c>
+      <c r="D195" t="s">
+        <v>190</v>
+      </c>
+      <c r="E195" t="s">
+        <v>60</v>
+      </c>
+      <c r="F195" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="196" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A196" t="s">
+        <v>212</v>
+      </c>
+      <c r="B196" t="s">
+        <v>213</v>
+      </c>
+      <c r="C196" t="s">
+        <v>54</v>
+      </c>
+      <c r="D196" t="s">
+        <v>191</v>
+      </c>
+      <c r="E196" t="s">
+        <v>192</v>
+      </c>
+      <c r="F196" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="197" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A197" t="s">
+        <v>212</v>
+      </c>
+      <c r="B197" t="s">
+        <v>213</v>
+      </c>
+      <c r="C197" t="s">
+        <v>54</v>
+      </c>
+      <c r="D197" t="s">
+        <v>193</v>
+      </c>
+      <c r="E197" t="s">
+        <v>194</v>
+      </c>
+      <c r="F197" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="198" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A198" t="s">
+        <v>212</v>
+      </c>
+      <c r="B198" t="s">
+        <v>213</v>
+      </c>
+      <c r="C198" t="s">
+        <v>54</v>
+      </c>
+      <c r="D198" t="s">
+        <v>195</v>
+      </c>
+      <c r="E198" t="s">
+        <v>196</v>
+      </c>
+      <c r="F198" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="199" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A199" t="s">
+        <v>212</v>
+      </c>
+      <c r="B199" t="s">
+        <v>213</v>
+      </c>
+      <c r="C199" t="s">
+        <v>54</v>
+      </c>
+      <c r="D199" t="s">
+        <v>197</v>
+      </c>
+      <c r="E199" t="s">
+        <v>198</v>
+      </c>
+      <c r="F199" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="200" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A200" t="s">
+        <v>212</v>
+      </c>
+      <c r="B200" t="s">
+        <v>213</v>
+      </c>
+      <c r="C200" t="s">
+        <v>54</v>
+      </c>
+      <c r="D200" t="s">
+        <v>199</v>
+      </c>
+      <c r="E200" t="s">
+        <v>200</v>
+      </c>
+      <c r="F200" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="201" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A201" t="s">
+        <v>212</v>
+      </c>
+      <c r="B201" t="s">
+        <v>213</v>
+      </c>
+      <c r="C201" t="s">
+        <v>54</v>
+      </c>
+      <c r="D201" t="s">
+        <v>201</v>
+      </c>
+      <c r="E201" t="s">
+        <v>202</v>
+      </c>
+      <c r="F201" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="202" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A202" t="s">
+        <v>212</v>
+      </c>
+      <c r="B202" t="s">
+        <v>213</v>
+      </c>
+      <c r="C202" t="s">
+        <v>54</v>
+      </c>
+      <c r="D202" t="s">
+        <v>203</v>
+      </c>
+      <c r="E202" t="s">
+        <v>204</v>
+      </c>
+      <c r="F202" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="203" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A203" t="s">
+        <v>212</v>
+      </c>
+      <c r="B203" t="s">
+        <v>213</v>
+      </c>
+      <c r="C203" t="s">
+        <v>54</v>
+      </c>
+      <c r="D203" t="s">
+        <v>205</v>
+      </c>
+      <c r="E203" t="s">
+        <v>206</v>
+      </c>
+      <c r="F203" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="204" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A204" t="s">
+        <v>212</v>
+      </c>
+      <c r="B204" t="s">
+        <v>213</v>
+      </c>
+      <c r="C204" t="s">
+        <v>54</v>
+      </c>
+      <c r="D204" t="s">
+        <v>207</v>
+      </c>
+      <c r="E204" t="s">
+        <v>208</v>
+      </c>
+      <c r="F204" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="205" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A205" t="s">
+        <v>214</v>
+      </c>
+      <c r="B205" t="s">
+        <v>215</v>
+      </c>
+      <c r="C205" t="s">
+        <v>16</v>
+      </c>
+      <c r="D205" t="s">
+        <v>18</v>
+      </c>
+      <c r="E205" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="206" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A206" t="s">
+        <v>214</v>
+      </c>
+      <c r="B206" t="s">
+        <v>215</v>
+      </c>
+      <c r="C206" t="s">
+        <v>19</v>
+      </c>
+      <c r="D206" t="s">
+        <v>65</v>
+      </c>
+      <c r="E206" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="207" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A207" t="s">
+        <v>214</v>
+      </c>
+      <c r="B207" t="s">
+        <v>215</v>
+      </c>
+      <c r="C207" t="s">
+        <v>66</v>
+      </c>
+      <c r="D207" t="s">
+        <v>22</v>
+      </c>
+      <c r="E207" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="208" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A208" t="s">
+        <v>214</v>
+      </c>
+      <c r="B208" t="s">
+        <v>215</v>
+      </c>
+      <c r="C208" t="s">
+        <v>66</v>
+      </c>
+      <c r="D208" t="s">
+        <v>67</v>
+      </c>
+      <c r="E208" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="209" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A209" t="s">
+        <v>214</v>
+      </c>
+      <c r="B209" t="s">
+        <v>215</v>
+      </c>
+      <c r="C209" t="s">
+        <v>66</v>
+      </c>
+      <c r="D209" t="s">
+        <v>23</v>
+      </c>
+      <c r="E209" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="210" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A210" t="s">
+        <v>214</v>
+      </c>
+      <c r="B210" t="s">
+        <v>215</v>
+      </c>
+      <c r="C210" t="s">
+        <v>89</v>
+      </c>
+      <c r="D210" t="s">
+        <v>186</v>
+      </c>
+      <c r="E210" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="211" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A211" t="s">
+        <v>214</v>
+      </c>
+      <c r="B211" t="s">
+        <v>215</v>
+      </c>
+      <c r="C211" t="s">
+        <v>54</v>
+      </c>
+      <c r="D211" t="s">
+        <v>187</v>
+      </c>
+      <c r="E211" t="s">
+        <v>188</v>
+      </c>
+      <c r="F211" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="212" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A212" t="s">
+        <v>214</v>
+      </c>
+      <c r="B212" t="s">
+        <v>215</v>
+      </c>
+      <c r="C212" t="s">
+        <v>54</v>
+      </c>
+      <c r="D212" t="s">
+        <v>190</v>
+      </c>
+      <c r="E212" t="s">
+        <v>60</v>
+      </c>
+      <c r="F212" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="213" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A213" t="s">
+        <v>214</v>
+      </c>
+      <c r="B213" t="s">
+        <v>215</v>
+      </c>
+      <c r="C213" t="s">
+        <v>54</v>
+      </c>
+      <c r="D213" t="s">
+        <v>191</v>
+      </c>
+      <c r="E213" t="s">
+        <v>192</v>
+      </c>
+      <c r="F213" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="214" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A214" t="s">
+        <v>214</v>
+      </c>
+      <c r="B214" t="s">
+        <v>215</v>
+      </c>
+      <c r="C214" t="s">
+        <v>54</v>
+      </c>
+      <c r="D214" t="s">
+        <v>193</v>
+      </c>
+      <c r="E214" t="s">
+        <v>194</v>
+      </c>
+      <c r="F214" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="215" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A215" t="s">
+        <v>214</v>
+      </c>
+      <c r="B215" t="s">
+        <v>215</v>
+      </c>
+      <c r="C215" t="s">
+        <v>54</v>
+      </c>
+      <c r="D215" t="s">
+        <v>195</v>
+      </c>
+      <c r="E215" t="s">
+        <v>196</v>
+      </c>
+      <c r="F215" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="216" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A216" t="s">
+        <v>214</v>
+      </c>
+      <c r="B216" t="s">
+        <v>215</v>
+      </c>
+      <c r="C216" t="s">
+        <v>54</v>
+      </c>
+      <c r="D216" t="s">
+        <v>197</v>
+      </c>
+      <c r="E216" t="s">
+        <v>198</v>
+      </c>
+      <c r="F216" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="217" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A217" t="s">
+        <v>214</v>
+      </c>
+      <c r="B217" t="s">
+        <v>215</v>
+      </c>
+      <c r="C217" t="s">
+        <v>54</v>
+      </c>
+      <c r="D217" t="s">
+        <v>199</v>
+      </c>
+      <c r="E217" t="s">
+        <v>200</v>
+      </c>
+      <c r="F217" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="218" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A218" t="s">
+        <v>214</v>
+      </c>
+      <c r="B218" t="s">
+        <v>215</v>
+      </c>
+      <c r="C218" t="s">
+        <v>54</v>
+      </c>
+      <c r="D218" t="s">
+        <v>201</v>
+      </c>
+      <c r="E218" t="s">
+        <v>202</v>
+      </c>
+      <c r="F218" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="219" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A219" t="s">
+        <v>214</v>
+      </c>
+      <c r="B219" t="s">
+        <v>215</v>
+      </c>
+      <c r="C219" t="s">
+        <v>54</v>
+      </c>
+      <c r="D219" t="s">
+        <v>203</v>
+      </c>
+      <c r="E219" t="s">
+        <v>204</v>
+      </c>
+      <c r="F219" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="220" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A220" t="s">
+        <v>214</v>
+      </c>
+      <c r="B220" t="s">
+        <v>215</v>
+      </c>
+      <c r="C220" t="s">
+        <v>54</v>
+      </c>
+      <c r="D220" t="s">
+        <v>205</v>
+      </c>
+      <c r="E220" t="s">
+        <v>206</v>
+      </c>
+      <c r="F220" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="221" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A221" t="s">
+        <v>214</v>
+      </c>
+      <c r="B221" t="s">
+        <v>215</v>
+      </c>
+      <c r="C221" t="s">
+        <v>54</v>
+      </c>
+      <c r="D221" t="s">
+        <v>207</v>
+      </c>
+      <c r="E221" t="s">
+        <v>208</v>
+      </c>
+      <c r="F221" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="222" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A222" t="s">
+        <v>216</v>
+      </c>
+      <c r="B222" t="s">
+        <v>217</v>
+      </c>
+      <c r="C222" t="s">
+        <v>16</v>
+      </c>
+      <c r="D222" t="s">
+        <v>18</v>
+      </c>
+      <c r="E222" t="s">
+        <v>18</v>
+      </c>
+      <c r="F222" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="223" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A223" t="s">
+        <v>216</v>
+      </c>
+      <c r="B223" t="s">
+        <v>217</v>
+      </c>
+      <c r="C223" t="s">
+        <v>66</v>
+      </c>
+      <c r="D223" t="s">
+        <v>22</v>
+      </c>
+      <c r="E223" t="s">
+        <v>22</v>
+      </c>
+      <c r="F223" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="224" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A224" t="s">
+        <v>216</v>
+      </c>
+      <c r="B224" t="s">
+        <v>217</v>
+      </c>
+      <c r="C224" t="s">
+        <v>66</v>
+      </c>
+      <c r="D224" t="s">
+        <v>23</v>
+      </c>
+      <c r="E224" t="s">
+        <v>23</v>
+      </c>
+      <c r="F224" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="225" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A225" t="s">
+        <v>216</v>
+      </c>
+      <c r="B225" t="s">
+        <v>217</v>
+      </c>
+      <c r="C225" t="s">
+        <v>89</v>
+      </c>
+      <c r="D225" t="s">
+        <v>186</v>
+      </c>
+      <c r="E225" t="s">
+        <v>186</v>
+      </c>
+      <c r="F225" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="226" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A226" t="s">
+        <v>216</v>
+      </c>
+      <c r="B226" t="s">
+        <v>217</v>
+      </c>
+      <c r="C226" t="s">
+        <v>54</v>
+      </c>
+      <c r="D226" t="s">
+        <v>187</v>
+      </c>
+      <c r="E226" t="s">
+        <v>188</v>
+      </c>
+      <c r="F226" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="227" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A227" t="s">
+        <v>216</v>
+      </c>
+      <c r="B227" t="s">
+        <v>217</v>
+      </c>
+      <c r="C227" t="s">
+        <v>54</v>
+      </c>
+      <c r="D227" t="s">
+        <v>190</v>
+      </c>
+      <c r="E227" t="s">
+        <v>60</v>
+      </c>
+      <c r="F227" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="228" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A228" t="s">
+        <v>216</v>
+      </c>
+      <c r="B228" t="s">
+        <v>217</v>
+      </c>
+      <c r="C228" t="s">
+        <v>54</v>
+      </c>
+      <c r="D228" t="s">
+        <v>191</v>
+      </c>
+      <c r="E228" t="s">
+        <v>192</v>
+      </c>
+      <c r="F228" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="229" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A229" t="s">
+        <v>216</v>
+      </c>
+      <c r="B229" t="s">
+        <v>217</v>
+      </c>
+      <c r="C229" t="s">
+        <v>54</v>
+      </c>
+      <c r="D229" t="s">
+        <v>193</v>
+      </c>
+      <c r="E229" t="s">
+        <v>194</v>
+      </c>
+      <c r="F229" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="230" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A230" t="s">
+        <v>216</v>
+      </c>
+      <c r="B230" t="s">
+        <v>217</v>
+      </c>
+      <c r="C230" t="s">
+        <v>54</v>
+      </c>
+      <c r="D230" t="s">
+        <v>195</v>
+      </c>
+      <c r="E230" t="s">
+        <v>196</v>
+      </c>
+      <c r="F230" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="231" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A231" t="s">
+        <v>216</v>
+      </c>
+      <c r="B231" t="s">
+        <v>217</v>
+      </c>
+      <c r="C231" t="s">
+        <v>54</v>
+      </c>
+      <c r="D231" t="s">
+        <v>197</v>
+      </c>
+      <c r="E231" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="232" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A232" t="s">
+        <v>216</v>
+      </c>
+      <c r="B232" t="s">
+        <v>217</v>
+      </c>
+      <c r="C232" t="s">
+        <v>54</v>
+      </c>
+      <c r="D232" t="s">
+        <v>199</v>
+      </c>
+      <c r="E232" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="233" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A233" t="s">
+        <v>216</v>
+      </c>
+      <c r="B233" t="s">
+        <v>217</v>
+      </c>
+      <c r="C233" t="s">
+        <v>54</v>
+      </c>
+      <c r="D233" t="s">
+        <v>201</v>
+      </c>
+      <c r="E233" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="234" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A234" t="s">
+        <v>216</v>
+      </c>
+      <c r="B234" t="s">
+        <v>217</v>
+      </c>
+      <c r="C234" t="s">
+        <v>54</v>
+      </c>
+      <c r="D234" t="s">
+        <v>203</v>
+      </c>
+      <c r="E234" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="235" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A235" t="s">
+        <v>216</v>
+      </c>
+      <c r="B235" t="s">
+        <v>217</v>
+      </c>
+      <c r="C235" t="s">
+        <v>54</v>
+      </c>
+      <c r="D235" t="s">
+        <v>205</v>
+      </c>
+      <c r="E235" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="236" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A236" t="s">
+        <v>216</v>
+      </c>
+      <c r="B236" t="s">
+        <v>217</v>
+      </c>
+      <c r="C236" t="s">
+        <v>54</v>
+      </c>
+      <c r="D236" t="s">
+        <v>207</v>
+      </c>
+      <c r="E236" t="s">
+        <v>208</v>
+      </c>
+      <c r="F236" t="s">
+        <v>189</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Aggiornati excel con nuovi file e aggiornamenti di precedentemente analizzati
</commit_message>
<xml_diff>
--- a/WP-2/Data_cleaning/ADNI_variables_cleaned1_COPIA.xlsx
+++ b/WP-2/Data_cleaning/ADNI_variables_cleaned1_COPIA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ifabfoundation-my.sharepoint.com/personal/chiara_pollicini_ifabfoundation_org/Documents/Documenti/Github/AIND/WP-2/Data_cleaning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{58F97C13-2200-4528-B3C3-FAD4C4233A7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F5165C9-DD69-4735-BF09-1E8E90475AC3}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{58F97C13-2200-4528-B3C3-FAD4C4233A7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD299DB8-A4D3-4288-B9A3-691F0684065C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4980" yWindow="-16680" windowWidth="28800" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2334" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2510" uniqueCount="271">
   <si>
     <t>file_name</t>
   </si>
@@ -717,6 +717,135 @@
   </si>
   <si>
     <t>ABETA42</t>
+  </si>
+  <si>
+    <t>The DIAN-ADNI Comparison Study</t>
+  </si>
+  <si>
+    <t>ADNI_DIAN_COMPARISON</t>
+  </si>
+  <si>
+    <t>VISCODE</t>
+  </si>
+  <si>
+    <t>BIRTHYR</t>
+  </si>
+  <si>
+    <t>CDRGLOB</t>
+  </si>
+  <si>
+    <t>CDRSUM</t>
+  </si>
+  <si>
+    <t>CDR_BASELINE</t>
+  </si>
+  <si>
+    <t>CORT</t>
+  </si>
+  <si>
+    <t>CSFDATE</t>
+  </si>
+  <si>
+    <t>CSF_CDRSB_BL</t>
+  </si>
+  <si>
+    <t>CSF_CDR_BL</t>
+  </si>
+  <si>
+    <t>CSF_DATE_BL</t>
+  </si>
+  <si>
+    <t>CSF_ELC_AB40</t>
+  </si>
+  <si>
+    <t>CSF_ELC_AB42</t>
+  </si>
+  <si>
+    <t>CSF_ELC_AB4240</t>
+  </si>
+  <si>
+    <t>CSF_ELC_PTAU</t>
+  </si>
+  <si>
+    <t>CSF_ELC_TAU</t>
+  </si>
+  <si>
+    <t>DIAN_APOE</t>
+  </si>
+  <si>
+    <t>DIAN_CDRSB_BL</t>
+  </si>
+  <si>
+    <t>DIAN_MMSE</t>
+  </si>
+  <si>
+    <t>DIAN_YEARS_BL</t>
+  </si>
+  <si>
+    <t>LAST_VISIT_DATE</t>
+  </si>
+  <si>
+    <t>MARISTAT</t>
+  </si>
+  <si>
+    <t>MRI_CDRSB_BL</t>
+  </si>
+  <si>
+    <t>MRI_CDR_BL</t>
+  </si>
+  <si>
+    <t>MRI_DATE_BL</t>
+  </si>
+  <si>
+    <t>MRI_SCANDATE</t>
+  </si>
+  <si>
+    <t>MR_TOTT_PRECUNEUS</t>
+  </si>
+  <si>
+    <t>MR_TOTV_HIPPOCAMPUS</t>
+  </si>
+  <si>
+    <t>MR_TOTV_INTRACRANIAL</t>
+  </si>
+  <si>
+    <t>MR_TOTV_WMHYPOINTENSITIES</t>
+  </si>
+  <si>
+    <t>PET_CDRSB_BL</t>
+  </si>
+  <si>
+    <t>PET_CDR_BL</t>
+  </si>
+  <si>
+    <t>PET_DATE_BL</t>
+  </si>
+  <si>
+    <t>PET_SCANDATE</t>
+  </si>
+  <si>
+    <t>PET_TYPE</t>
+  </si>
+  <si>
+    <t>PIB_FSUVR_RSF_TOT_CORTMEAN</t>
+  </si>
+  <si>
+    <t>PIB_FSUVR_RSF_TOT_CTX_PRECUNEUS</t>
+  </si>
+  <si>
+    <t>PIB_FSUVR_RSF_TOT_HIPPOCAMPUS</t>
+  </si>
+  <si>
+    <t>PIB_MSUVR_TOT_CORTMEAN</t>
+  </si>
+  <si>
+    <t>PIB_MSUVR_TOT_PRECUNEUS</t>
+  </si>
+  <si>
+    <t>VISITAGE</t>
+  </si>
+  <si>
+    <t>VISIT_DATE_BL</t>
   </si>
 </sst>
 </file>
@@ -1089,10 +1218,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O283"/>
+  <dimension ref="A1:Y283"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1139,7 +1268,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1162,7 +1291,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -1184,8 +1313,20 @@
       <c r="M3" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V3" t="s">
+        <v>228</v>
+      </c>
+      <c r="W3" t="s">
+        <v>229</v>
+      </c>
+      <c r="X3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -1207,8 +1348,20 @@
       <c r="M4" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V4" t="s">
+        <v>228</v>
+      </c>
+      <c r="W4" t="s">
+        <v>229</v>
+      </c>
+      <c r="X4" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -1230,8 +1383,20 @@
       <c r="M5" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V5" t="s">
+        <v>228</v>
+      </c>
+      <c r="W5" t="s">
+        <v>229</v>
+      </c>
+      <c r="X5" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -1253,8 +1418,20 @@
       <c r="M6" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V6" t="s">
+        <v>228</v>
+      </c>
+      <c r="W6" t="s">
+        <v>229</v>
+      </c>
+      <c r="X6" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -1279,8 +1456,20 @@
       <c r="N7" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V7" t="s">
+        <v>228</v>
+      </c>
+      <c r="W7" t="s">
+        <v>229</v>
+      </c>
+      <c r="X7" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="8" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -1305,8 +1494,20 @@
       <c r="N8" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V8" t="s">
+        <v>228</v>
+      </c>
+      <c r="W8" t="s">
+        <v>229</v>
+      </c>
+      <c r="X8" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -1331,8 +1532,20 @@
       <c r="N9" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V9" t="s">
+        <v>228</v>
+      </c>
+      <c r="W9" t="s">
+        <v>229</v>
+      </c>
+      <c r="X9" t="s">
+        <v>82</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -1357,8 +1570,20 @@
       <c r="N10" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V10" t="s">
+        <v>228</v>
+      </c>
+      <c r="W10" t="s">
+        <v>229</v>
+      </c>
+      <c r="X10" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="11" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -1383,8 +1608,20 @@
       <c r="N11" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V11" t="s">
+        <v>228</v>
+      </c>
+      <c r="W11" t="s">
+        <v>229</v>
+      </c>
+      <c r="X11" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="12" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -1409,8 +1646,20 @@
       <c r="N12" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V12" t="s">
+        <v>228</v>
+      </c>
+      <c r="W12" t="s">
+        <v>229</v>
+      </c>
+      <c r="X12" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="13" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -1438,8 +1687,20 @@
       <c r="O13" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V13" t="s">
+        <v>228</v>
+      </c>
+      <c r="W13" t="s">
+        <v>229</v>
+      </c>
+      <c r="X13" t="s">
+        <v>82</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="14" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -1467,8 +1728,20 @@
       <c r="O14" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V14" t="s">
+        <v>228</v>
+      </c>
+      <c r="W14" t="s">
+        <v>229</v>
+      </c>
+      <c r="X14" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -1496,8 +1769,20 @@
       <c r="O15" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V15" t="s">
+        <v>228</v>
+      </c>
+      <c r="W15" t="s">
+        <v>229</v>
+      </c>
+      <c r="X15" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -1525,8 +1810,20 @@
       <c r="O16" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V16" t="s">
+        <v>228</v>
+      </c>
+      <c r="W16" t="s">
+        <v>229</v>
+      </c>
+      <c r="X16" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="17" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -1554,8 +1851,20 @@
       <c r="O17" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V17" t="s">
+        <v>228</v>
+      </c>
+      <c r="W17" t="s">
+        <v>229</v>
+      </c>
+      <c r="X17" t="s">
+        <v>71</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="18" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>14</v>
       </c>
@@ -1583,8 +1892,20 @@
       <c r="O18" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V18" t="s">
+        <v>228</v>
+      </c>
+      <c r="W18" t="s">
+        <v>229</v>
+      </c>
+      <c r="X18" t="s">
+        <v>71</v>
+      </c>
+      <c r="Y18" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="19" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>14</v>
       </c>
@@ -1612,8 +1933,20 @@
       <c r="O19" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V19" t="s">
+        <v>228</v>
+      </c>
+      <c r="W19" t="s">
+        <v>229</v>
+      </c>
+      <c r="X19" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="20" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>14</v>
       </c>
@@ -1641,8 +1974,20 @@
       <c r="O20" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V20" t="s">
+        <v>228</v>
+      </c>
+      <c r="W20" t="s">
+        <v>229</v>
+      </c>
+      <c r="X20" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="21" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>14</v>
       </c>
@@ -1670,8 +2015,20 @@
       <c r="O21" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V21" t="s">
+        <v>228</v>
+      </c>
+      <c r="W21" t="s">
+        <v>229</v>
+      </c>
+      <c r="X21" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="22" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>14</v>
       </c>
@@ -1699,8 +2056,20 @@
       <c r="O22" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V22" t="s">
+        <v>228</v>
+      </c>
+      <c r="W22" t="s">
+        <v>229</v>
+      </c>
+      <c r="X22" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="23" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>14</v>
       </c>
@@ -1728,8 +2097,20 @@
       <c r="O23" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V23" t="s">
+        <v>228</v>
+      </c>
+      <c r="W23" t="s">
+        <v>229</v>
+      </c>
+      <c r="X23" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="24" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>14</v>
       </c>
@@ -1757,8 +2138,20 @@
       <c r="O24" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V24" t="s">
+        <v>228</v>
+      </c>
+      <c r="W24" t="s">
+        <v>229</v>
+      </c>
+      <c r="X24" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="25" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>14</v>
       </c>
@@ -1786,8 +2179,20 @@
       <c r="O25" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V25" t="s">
+        <v>228</v>
+      </c>
+      <c r="W25" t="s">
+        <v>229</v>
+      </c>
+      <c r="X25" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="26" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>14</v>
       </c>
@@ -1815,8 +2220,20 @@
       <c r="O26" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V26" t="s">
+        <v>228</v>
+      </c>
+      <c r="W26" t="s">
+        <v>229</v>
+      </c>
+      <c r="X26" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y26" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="27" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>14</v>
       </c>
@@ -1844,8 +2261,20 @@
       <c r="O27" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V27" t="s">
+        <v>228</v>
+      </c>
+      <c r="W27" t="s">
+        <v>229</v>
+      </c>
+      <c r="X27" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y27" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="28" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>14</v>
       </c>
@@ -1867,8 +2296,20 @@
       <c r="M28" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V28" t="s">
+        <v>228</v>
+      </c>
+      <c r="W28" t="s">
+        <v>229</v>
+      </c>
+      <c r="X28" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y28" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="29" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>14</v>
       </c>
@@ -1890,8 +2331,20 @@
       <c r="M29" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V29" t="s">
+        <v>228</v>
+      </c>
+      <c r="W29" t="s">
+        <v>229</v>
+      </c>
+      <c r="X29" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y29" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="30" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>14</v>
       </c>
@@ -1910,8 +2363,20 @@
       <c r="M30" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V30" t="s">
+        <v>228</v>
+      </c>
+      <c r="W30" t="s">
+        <v>229</v>
+      </c>
+      <c r="X30" t="s">
+        <v>53</v>
+      </c>
+      <c r="Y30" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="31" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>62</v>
       </c>
@@ -1933,8 +2398,20 @@
       <c r="M31" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V31" t="s">
+        <v>228</v>
+      </c>
+      <c r="W31" t="s">
+        <v>229</v>
+      </c>
+      <c r="X31" t="s">
+        <v>53</v>
+      </c>
+      <c r="Y31" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="32" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>62</v>
       </c>
@@ -1956,8 +2433,20 @@
       <c r="M32" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V32" t="s">
+        <v>228</v>
+      </c>
+      <c r="W32" t="s">
+        <v>229</v>
+      </c>
+      <c r="X32" t="s">
+        <v>53</v>
+      </c>
+      <c r="Y32" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="33" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>62</v>
       </c>
@@ -1979,8 +2468,20 @@
       <c r="M33" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V33" t="s">
+        <v>228</v>
+      </c>
+      <c r="W33" t="s">
+        <v>229</v>
+      </c>
+      <c r="X33" t="s">
+        <v>53</v>
+      </c>
+      <c r="Y33" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="34" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>62</v>
       </c>
@@ -2002,8 +2503,20 @@
       <c r="M34" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V34" t="s">
+        <v>228</v>
+      </c>
+      <c r="W34" t="s">
+        <v>229</v>
+      </c>
+      <c r="X34" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y34" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="35" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>62</v>
       </c>
@@ -2028,8 +2541,20 @@
       <c r="N35" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V35" t="s">
+        <v>228</v>
+      </c>
+      <c r="W35" t="s">
+        <v>229</v>
+      </c>
+      <c r="X35" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y35" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="36" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>62</v>
       </c>
@@ -2054,8 +2579,20 @@
       <c r="N36" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V36" t="s">
+        <v>228</v>
+      </c>
+      <c r="W36" t="s">
+        <v>229</v>
+      </c>
+      <c r="X36" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y36" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="37" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>62</v>
       </c>
@@ -2080,8 +2617,20 @@
       <c r="N37" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V37" t="s">
+        <v>228</v>
+      </c>
+      <c r="W37" t="s">
+        <v>229</v>
+      </c>
+      <c r="X37" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y37" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="38" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>62</v>
       </c>
@@ -2106,8 +2655,20 @@
       <c r="N38" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V38" t="s">
+        <v>228</v>
+      </c>
+      <c r="W38" t="s">
+        <v>229</v>
+      </c>
+      <c r="X38" t="s">
+        <v>82</v>
+      </c>
+      <c r="Y38" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="39" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>62</v>
       </c>
@@ -2135,8 +2696,20 @@
       <c r="O39" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V39" t="s">
+        <v>228</v>
+      </c>
+      <c r="W39" t="s">
+        <v>229</v>
+      </c>
+      <c r="X39" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y39" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="40" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>62</v>
       </c>
@@ -2158,8 +2731,20 @@
       <c r="M40" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V40" t="s">
+        <v>228</v>
+      </c>
+      <c r="W40" t="s">
+        <v>229</v>
+      </c>
+      <c r="X40" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y40" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="41" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>62</v>
       </c>
@@ -2187,8 +2772,20 @@
       <c r="O41" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V41" t="s">
+        <v>228</v>
+      </c>
+      <c r="W41" t="s">
+        <v>229</v>
+      </c>
+      <c r="X41" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y41" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="42" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>62</v>
       </c>
@@ -2210,8 +2807,20 @@
       <c r="M42" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V42" t="s">
+        <v>228</v>
+      </c>
+      <c r="W42" t="s">
+        <v>229</v>
+      </c>
+      <c r="X42" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y42" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="43" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>62</v>
       </c>
@@ -2239,8 +2848,20 @@
       <c r="O43" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V43" t="s">
+        <v>228</v>
+      </c>
+      <c r="W43" t="s">
+        <v>229</v>
+      </c>
+      <c r="X43" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y43" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="44" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>62</v>
       </c>
@@ -2268,8 +2889,20 @@
       <c r="O44" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V44" t="s">
+        <v>228</v>
+      </c>
+      <c r="W44" t="s">
+        <v>229</v>
+      </c>
+      <c r="X44" t="s">
+        <v>30</v>
+      </c>
+      <c r="Y44" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="45" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>62</v>
       </c>
@@ -2297,8 +2930,20 @@
       <c r="O45" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V45" t="s">
+        <v>228</v>
+      </c>
+      <c r="W45" t="s">
+        <v>229</v>
+      </c>
+      <c r="X45" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y45" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="46" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>62</v>
       </c>
@@ -2326,8 +2971,20 @@
       <c r="O46" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="V46" t="s">
+        <v>228</v>
+      </c>
+      <c r="W46" t="s">
+        <v>229</v>
+      </c>
+      <c r="X46" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y46" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="47" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>62</v>
       </c>
@@ -2350,7 +3007,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>62</v>
       </c>

</xml_diff>